<commit_message>
80% json Vada + scripts stats et amélioration des json
</commit_message>
<xml_diff>
--- a/echantillon_llm_tagged.xlsx
+++ b/echantillon_llm_tagged.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\Project_Internship\Index_Insight\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C7DBFE-2076-4FC3-8CD6-84265D698660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25497A6-51AB-488A-A315-B21384F9D368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13759" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="112">
   <si>
     <t>Catégorie</t>
   </si>
@@ -1186,6 +1186,9 @@
   </si>
   <si>
     <t>Nature de l'initiative en plus ?</t>
+  </si>
+  <si>
+    <t>Peut etre le cout de l'initiative</t>
   </si>
 </sst>
 </file>
@@ -1591,7 +1594,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" style="1" bestFit="1" customWidth="1"/>
@@ -2053,6 +2056,11 @@
         <v>110</v>
       </c>
     </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>